<commit_message>
Atualiza dados do painel
</commit_message>
<xml_diff>
--- a/public/Dados_copese.xlsx
+++ b/public/Dados_copese.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leonardo\sisu-ufpi-dashboard\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E2693AA-4DE2-44BA-865D-A72BF59D9C7B}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4BAAB1F-4D10-40ED-9301-CB51D52F844A}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vagas" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14418" uniqueCount="1603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14418" uniqueCount="1602">
   <si>
     <t>ano_s</t>
   </si>
@@ -4837,9 +4837,6 @@
   </si>
   <si>
     <t>Matrícula Indeferida</t>
-  </si>
-  <si>
-    <t>Aguardando matrícula</t>
   </si>
   <si>
     <t>ND</t>
@@ -4849,11 +4846,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -4939,32 +4943,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -7370,11 +7375,11 @@
   convocacoes!E:E, F60,
   convocacoes!I:I, 1
 )</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I60" s="2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7442,11 +7447,11 @@
   convocacoes!E:E, F62,
   convocacoes!I:I, 1
 )</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I62" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7478,11 +7483,11 @@
   convocacoes!E:E, F63,
   convocacoes!I:I, 1
 )</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I63" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7514,11 +7519,11 @@
   convocacoes!E:E, F64,
   convocacoes!I:I, 1
 )</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I64" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7550,11 +7555,11 @@
   convocacoes!E:E, F65,
   convocacoes!I:I, 1
 )</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I65" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7622,11 +7627,11 @@
   convocacoes!E:E, F67,
   convocacoes!I:I, 1
 )</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I67" s="2">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7694,11 +7699,11 @@
   convocacoes!E:E, F69,
   convocacoes!I:I, 1
 )</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I69" s="2">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -8628,7 +8633,7 @@
     <row r="994" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <autoFilter ref="A1:I59" xr:uid="{757EA66F-DC97-48A0-A498-5FBE3B3AA156}"/>
-  <phoneticPr fontId="9" type="noConversion"/>
+  <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -14201,7 +14206,7 @@
         <v>50</v>
       </c>
       <c r="L158" s="19" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="159" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -14237,7 +14242,7 @@
       </c>
       <c r="K159" s="4"/>
       <c r="L159" s="19" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="160" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -14345,7 +14350,7 @@
       </c>
       <c r="K162" s="4"/>
       <c r="L162" s="19" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="163" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -14453,7 +14458,7 @@
       </c>
       <c r="K165" s="4"/>
       <c r="L165" s="19" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="166" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -14527,7 +14532,7 @@
         <v>1582</v>
       </c>
       <c r="L167" s="19" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="168" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -14599,7 +14604,7 @@
       </c>
       <c r="K169" s="4"/>
       <c r="L169" s="19" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="170" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -14635,7 +14640,7 @@
       </c>
       <c r="K170" s="4"/>
       <c r="L170" s="19" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="171" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -14671,7 +14676,7 @@
       </c>
       <c r="K171" s="4"/>
       <c r="L171" s="19" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="172" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -14747,7 +14752,7 @@
         <v>789</v>
       </c>
       <c r="L173" s="19" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="174" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -14785,7 +14790,7 @@
         <v>789</v>
       </c>
       <c r="L174" s="19" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="175" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -14823,7 +14828,7 @@
         <v>789</v>
       </c>
       <c r="L175" s="19" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="176" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -14854,8 +14859,8 @@
       <c r="I176" s="4">
         <v>0</v>
       </c>
-      <c r="J176" s="19" t="s">
-        <v>1601</v>
+      <c r="J176" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="L176" s="18" t="s">
         <v>88</v>
@@ -14887,10 +14892,10 @@
         <v>1137</v>
       </c>
       <c r="I177" s="4">
-        <v>0</v>
-      </c>
-      <c r="J177" s="19" t="s">
-        <v>1601</v>
+        <v>1</v>
+      </c>
+      <c r="J177" s="20" t="s">
+        <v>70</v>
       </c>
       <c r="K177" s="19" t="s">
         <v>25</v>
@@ -14927,8 +14932,8 @@
       <c r="I178" s="4">
         <v>0</v>
       </c>
-      <c r="J178" s="19" t="s">
-        <v>1601</v>
+      <c r="J178" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="K178" s="19" t="s">
         <v>789</v>
@@ -14963,10 +14968,10 @@
         <v>1140</v>
       </c>
       <c r="I179" s="4">
-        <v>0</v>
-      </c>
-      <c r="J179" s="19" t="s">
-        <v>1601</v>
+        <v>1</v>
+      </c>
+      <c r="J179" s="20" t="s">
+        <v>70</v>
       </c>
       <c r="K179" s="19" t="s">
         <v>25</v>
@@ -15001,13 +15006,13 @@
         <v>101</v>
       </c>
       <c r="I180" s="4">
-        <v>0</v>
-      </c>
-      <c r="J180" s="19" t="s">
-        <v>1601</v>
-      </c>
-      <c r="L180" s="18" t="s">
-        <v>88</v>
+        <v>1</v>
+      </c>
+      <c r="J180" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="L180" t="s">
+        <v>1594</v>
       </c>
     </row>
     <row r="181" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -15038,8 +15043,8 @@
       <c r="I181" s="4">
         <v>0</v>
       </c>
-      <c r="J181" s="19" t="s">
-        <v>1601</v>
+      <c r="J181" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="L181" s="18" t="s">
         <v>88</v>
@@ -15071,13 +15076,13 @@
         <v>651</v>
       </c>
       <c r="I182" s="4">
-        <v>0</v>
-      </c>
-      <c r="J182" s="19" t="s">
-        <v>1601</v>
-      </c>
-      <c r="L182" s="18" t="s">
-        <v>88</v>
+        <v>1</v>
+      </c>
+      <c r="J182" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="L182" t="s">
+        <v>1594</v>
       </c>
     </row>
     <row r="183" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -15106,13 +15111,13 @@
         <v>107</v>
       </c>
       <c r="I183" s="4">
-        <v>0</v>
-      </c>
-      <c r="J183" s="19" t="s">
-        <v>1601</v>
-      </c>
-      <c r="L183" s="18" t="s">
-        <v>88</v>
+        <v>1</v>
+      </c>
+      <c r="J183" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="L183" t="s">
+        <v>1594</v>
       </c>
     </row>
     <row r="184" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -15141,10 +15146,10 @@
         <v>1217</v>
       </c>
       <c r="I184" s="4">
-        <v>0</v>
-      </c>
-      <c r="J184" s="19" t="s">
-        <v>1601</v>
+        <v>1</v>
+      </c>
+      <c r="J184" s="20" t="s">
+        <v>70</v>
       </c>
       <c r="L184" s="18" t="s">
         <v>88</v>
@@ -15176,10 +15181,10 @@
         <v>1276</v>
       </c>
       <c r="I185" s="4">
-        <v>0</v>
-      </c>
-      <c r="J185" s="19" t="s">
-        <v>1601</v>
+        <v>1</v>
+      </c>
+      <c r="J185" s="20" t="s">
+        <v>70</v>
       </c>
       <c r="K185" s="19" t="s">
         <v>1582</v>
@@ -15214,10 +15219,10 @@
         <v>1297</v>
       </c>
       <c r="I186" s="4">
-        <v>0</v>
-      </c>
-      <c r="J186" s="19" t="s">
-        <v>1601</v>
+        <v>1</v>
+      </c>
+      <c r="J186" s="20" t="s">
+        <v>70</v>
       </c>
       <c r="K186" s="19" t="s">
         <v>1582</v>
@@ -15228,7 +15233,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L186" xr:uid="{DCF350D5-A937-4A0D-B6AA-DEB16DD30D95}"/>
-  <phoneticPr fontId="9" type="noConversion"/>
+  <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>

</xml_diff>